<commit_message>
Electronics BOM without links
</commit_message>
<xml_diff>
--- a/1_ORGO-15_P1/BOM_ORGO-15_P1.xlsx
+++ b/1_ORGO-15_P1/BOM_ORGO-15_P1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-Model\1_ORGO-15_P1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ORGOfly\ORGOfly-CAD-model\1_ORGO-15_P1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F19D5243-48B3-478D-B86C-F33AF1F8935E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{907A97BC-A127-40F9-90B8-4234044E0AF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Background_info" sheetId="2" state="hidden" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="113">
   <si>
     <t>#</t>
   </si>
@@ -237,13 +237,154 @@
   </si>
   <si>
     <t>1kg - White!</t>
+  </si>
+  <si>
+    <t>Antenna</t>
+  </si>
+  <si>
+    <t>Multiple-cell battery</t>
+  </si>
+  <si>
+    <t>Unpolarized capacitor</t>
+  </si>
+  <si>
+    <t>SQESC_12100</t>
+  </si>
+  <si>
+    <t>HGLRC_M100_Pro</t>
+  </si>
+  <si>
+    <t>XT-90F</t>
+  </si>
+  <si>
+    <t>4mm_Banana_Conn_Socket</t>
+  </si>
+  <si>
+    <t>4mm_Banana_Conn_Pin</t>
+  </si>
+  <si>
+    <t>JST-SH1.0-8P_F</t>
+  </si>
+  <si>
+    <t>JST connector, single row, 01x08, SH 1.0</t>
+  </si>
+  <si>
+    <t>JST-SH1.0-8P_M</t>
+  </si>
+  <si>
+    <t>JST connector, single row, 01x08, Sh 1.0</t>
+  </si>
+  <si>
+    <t>JST-SH1.0-4P_F</t>
+  </si>
+  <si>
+    <t>JST connector, single row, 01x04</t>
+  </si>
+  <si>
+    <t>JST-SH1.0-4P_M</t>
+  </si>
+  <si>
+    <t>JST-SH1.0-6P_F</t>
+  </si>
+  <si>
+    <t>JST connector, single row, 01x06, SH 1.0</t>
+  </si>
+  <si>
+    <t>JST-SH1.0-6P_M</t>
+  </si>
+  <si>
+    <t>JST connector, single row, 01x06, SH1.0</t>
+  </si>
+  <si>
+    <t>MG996R</t>
+  </si>
+  <si>
+    <t>Servo Motor (JR connector)</t>
+  </si>
+  <si>
+    <t>Brotherhobby Avenger 3120 500KV</t>
+  </si>
+  <si>
+    <t>370 uF capacitor</t>
+  </si>
+  <si>
+    <t>Turnigy_HD_6S_5Ah5_60C_LiPo</t>
+  </si>
+  <si>
+    <t>Foxeer Mini Cat 4 1200TVL</t>
+  </si>
+  <si>
+    <t>FPV Camera</t>
+  </si>
+  <si>
+    <t>Power connector</t>
+  </si>
+  <si>
+    <t>JR connector, single row, 01x03</t>
+  </si>
+  <si>
+    <t>JR-3P_F</t>
+  </si>
+  <si>
+    <t>JR-3P_M</t>
+  </si>
+  <si>
+    <t>Mini Servo</t>
+  </si>
+  <si>
+    <t>Motor</t>
+  </si>
+  <si>
+    <t>TBS Crossfire Diversity Nano Rx</t>
+  </si>
+  <si>
+    <t>FPV LONG RANGE DRONE RECEIVER</t>
+  </si>
+  <si>
+    <t>ULTRA 25-1600mW 4.9-5.8G 64CH</t>
+  </si>
+  <si>
+    <t>MATEKSYS XCLAS PDB FCHUB-12S</t>
+  </si>
+  <si>
+    <t>Power Distribution Board</t>
+  </si>
+  <si>
+    <t>GPS with Compass</t>
+  </si>
+  <si>
+    <t>MATEKSYS_F405-HDTE  12 PWM</t>
+  </si>
+  <si>
+    <t>Flight Controller</t>
+  </si>
+  <si>
+    <t>Electronic Speed Controller</t>
+  </si>
+  <si>
+    <t>XT-90M</t>
+  </si>
+  <si>
+    <t>Video Transmitter</t>
+  </si>
+  <si>
+    <t>https://hobbyking.com/en_us/turnigy-heavy-duty-5500mah-6s-60c-lipo-pack-w-xt90.html</t>
+  </si>
+  <si>
+    <t>https://n-factory.de/F405-WING_15?srsltid=AfmBOorJLigbjhDd51Re4u0jHc0Jw6epVL2ePDy3WgvZ8yOpSwySAvJh</t>
+  </si>
+  <si>
+    <t>Sold in bulk</t>
+  </si>
+  <si>
+    <t>https://sequremall.com/products/sequre-12100-brushless-electric-speed-controller-5-12s-power-supply-100a-blheli_32-am32-firmware-support-128khz-pwm-frequency-suitable-for-multi-rotor-aircrafts-airplane-models-plant-protection-machine-boat-models-rc-car-models?srsltid=AfmBOoqD3cKLbLKnMnpXxBff0019A01XQKeqCUJ8P-pC8NoTSW-f13nF</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,6 +420,21 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="204"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -364,7 +520,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -420,6 +576,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -762,12 +924,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -778,7 +940,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -789,7 +951,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -800,7 +962,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -811,7 +973,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -822,7 +984,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -830,37 +992,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -872,31 +1034,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:M26"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:M35"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.77734375" style="7" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="57.77734375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="25.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="8.88671875" style="1"/>
-    <col min="8" max="8" width="4.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.21875" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="1"/>
+    <col min="2" max="2" width="37.7109375" style="7" customWidth="1"/>
+    <col min="3" max="3" width="57.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.85546875" style="1"/>
+    <col min="8" max="8" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" style="1"/>
     <col min="13" max="13" width="48" style="17" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="2"/>
+    <col min="14" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -937,7 +1099,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -974,7 +1136,7 @@
       </c>
       <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
@@ -1017,7 +1179,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
@@ -1060,7 +1222,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
@@ -1090,7 +1252,7 @@
         <v>44</v>
       </c>
       <c r="J6" s="15">
-        <f t="shared" ref="J6:J26" si="0">(G6*E6)+F6</f>
+        <f t="shared" ref="J6:J27" si="0">(G6*E6)+F6</f>
         <v>20.399999999999999</v>
       </c>
       <c r="K6" s="15" t="s">
@@ -1103,7 +1265,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
@@ -1146,7 +1308,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
@@ -1189,7 +1351,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
@@ -1228,7 +1390,7 @@
       </c>
       <c r="M9" s="16"/>
     </row>
-    <row r="10" spans="1:13" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
@@ -1271,17 +1433,25 @@
         <v>63</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="15" t="str">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
-        <v/>
-      </c>
-      <c r="B11" s="14"/>
-      <c r="C11" s="13"/>
-      <c r="D11" s="15"/>
+        <v>9</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>28</v>
+      </c>
       <c r="E11" s="15"/>
       <c r="F11" s="15"/>
-      <c r="G11" s="15"/>
+      <c r="G11" s="15">
+        <v>1</v>
+      </c>
       <c r="H11" s="15"/>
       <c r="I11" s="3"/>
       <c r="J11" s="15">
@@ -1289,41 +1459,67 @@
         <v>0</v>
       </c>
       <c r="K11" s="15"/>
-      <c r="L11" s="18"/>
+      <c r="L11" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M11" s="16"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="15" t="str">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A12" s="15">
         <f>IF(B12&lt;&gt;"",COUNTA($B$3:B12),"")</f>
-        <v/>
-      </c>
-      <c r="B12" s="14"/>
-      <c r="C12" s="13"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
+        <v>10</v>
+      </c>
+      <c r="B12" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D12" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="15">
+        <v>60.75</v>
+      </c>
       <c r="F12" s="15"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="3"/>
+      <c r="G12" s="15">
+        <v>4</v>
+      </c>
+      <c r="H12" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>109</v>
+      </c>
       <c r="J12" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>243</v>
       </c>
       <c r="K12" s="15"/>
-      <c r="L12" s="18"/>
+      <c r="L12" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M12" s="16"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A13" s="15" t="str">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A13" s="15">
         <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
-        <v/>
-      </c>
-      <c r="B13" s="14"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="15"/>
+        <v>11</v>
+      </c>
+      <c r="B13" s="14" t="s">
+        <v>88</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>68</v>
+      </c>
+      <c r="D13" s="15" t="s">
+        <v>19</v>
+      </c>
       <c r="E13" s="15"/>
       <c r="F13" s="15"/>
-      <c r="G13" s="15"/>
+      <c r="G13" s="15">
+        <v>1</v>
+      </c>
       <c r="H13" s="15"/>
       <c r="I13" s="3"/>
       <c r="J13" s="15">
@@ -1331,20 +1527,30 @@
         <v>0</v>
       </c>
       <c r="K13" s="15"/>
-      <c r="L13" s="18"/>
+      <c r="L13" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M13" s="16"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A14" s="15" t="str">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A14" s="15">
         <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
-        <v/>
-      </c>
-      <c r="B14" s="14"/>
-      <c r="C14" s="13"/>
-      <c r="D14" s="15"/>
+        <v>12</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
+      <c r="G14" s="15">
+        <v>1</v>
+      </c>
       <c r="H14" s="15"/>
       <c r="I14" s="3"/>
       <c r="J14" s="15">
@@ -1352,62 +1558,104 @@
         <v>0</v>
       </c>
       <c r="K14" s="15"/>
-      <c r="L14" s="18"/>
+      <c r="L14" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M14" s="16"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A15" s="15" t="str">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A15" s="15">
         <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
-        <v/>
-      </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
+        <v>13</v>
+      </c>
+      <c r="B15" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="D15" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E15" s="15">
+        <v>44.99</v>
+      </c>
       <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="3"/>
+      <c r="G15" s="15">
+        <v>4</v>
+      </c>
+      <c r="H15" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I15" s="3" t="s">
+        <v>112</v>
+      </c>
       <c r="J15" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>179.96</v>
       </c>
       <c r="K15" s="15"/>
-      <c r="L15" s="18"/>
+      <c r="L15" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M15" s="16"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="str">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A16" s="15">
         <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
-        <v/>
-      </c>
-      <c r="B16" s="14"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
+        <v>14</v>
+      </c>
+      <c r="B16" s="14" t="s">
+        <v>104</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="D16" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" s="15">
+        <v>49.95</v>
+      </c>
       <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="3"/>
+      <c r="G16" s="15">
+        <v>1</v>
+      </c>
+      <c r="H16" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I16" s="3" t="s">
+        <v>110</v>
+      </c>
       <c r="J16" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>49.95</v>
       </c>
       <c r="K16" s="15"/>
-      <c r="L16" s="18"/>
+      <c r="L16" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M16" s="16"/>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A17" s="15" t="str">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A17" s="15">
         <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
-        <v/>
-      </c>
-      <c r="B17" s="14"/>
-      <c r="C17" s="13"/>
-      <c r="D17" s="15"/>
+        <v>15</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>25</v>
+      </c>
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
-      <c r="G17" s="15"/>
+      <c r="G17" s="15">
+        <v>1</v>
+      </c>
       <c r="H17" s="15"/>
       <c r="I17" s="3"/>
       <c r="J17" s="15">
@@ -1415,20 +1663,30 @@
         <v>0</v>
       </c>
       <c r="K17" s="15"/>
-      <c r="L17" s="18"/>
+      <c r="L17" s="18" t="s">
+        <v>36</v>
+      </c>
       <c r="M17" s="16"/>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A18" s="15" t="str">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A18" s="15">
         <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
-        <v/>
-      </c>
-      <c r="B18" s="14"/>
-      <c r="C18" s="13"/>
-      <c r="D18" s="15"/>
+        <v>16</v>
+      </c>
+      <c r="B18" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E18" s="15"/>
       <c r="F18" s="15"/>
-      <c r="G18" s="15"/>
+      <c r="G18" s="15">
+        <v>8</v>
+      </c>
       <c r="H18" s="15"/>
       <c r="I18" s="3"/>
       <c r="J18" s="15">
@@ -1436,41 +1694,62 @@
         <v>0</v>
       </c>
       <c r="K18" s="15"/>
-      <c r="L18" s="18"/>
-      <c r="M18" s="16"/>
-    </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A19" s="15" t="str">
+      <c r="L18" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="15">
         <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
-        <v/>
-      </c>
-      <c r="B19" s="14"/>
-      <c r="C19" s="13"/>
-      <c r="D19" s="15"/>
+        <v>17</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>107</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D19" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E19" s="15"/>
       <c r="F19" s="15"/>
-      <c r="G19" s="15"/>
+      <c r="G19" s="15">
+        <v>8</v>
+      </c>
       <c r="H19" s="15"/>
       <c r="I19" s="3"/>
-      <c r="J19" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
+      <c r="J19" s="15"/>
       <c r="K19" s="15"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="16"/>
-    </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A20" s="15" t="str">
+      <c r="L19" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="15">
         <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
-        <v/>
-      </c>
-      <c r="B20" s="14"/>
-      <c r="C20" s="13"/>
-      <c r="D20" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D20" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E20" s="15"/>
       <c r="F20" s="15"/>
-      <c r="G20" s="15"/>
+      <c r="G20" s="15">
+        <v>12</v>
+      </c>
       <c r="H20" s="15"/>
       <c r="I20" s="3"/>
       <c r="J20" s="15">
@@ -1478,20 +1757,32 @@
         <v>0</v>
       </c>
       <c r="K20" s="15"/>
-      <c r="L20" s="18"/>
-      <c r="M20" s="16"/>
-    </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A21" s="15" t="str">
+      <c r="L20" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="15">
         <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
-        <v/>
-      </c>
-      <c r="B21" s="14"/>
-      <c r="C21" s="13"/>
-      <c r="D21" s="15"/>
+        <v>19</v>
+      </c>
+      <c r="B21" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="D21" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E21" s="15"/>
       <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
+      <c r="G21" s="15">
+        <v>12</v>
+      </c>
       <c r="H21" s="15"/>
       <c r="I21" s="3"/>
       <c r="J21" s="15">
@@ -1499,20 +1790,32 @@
         <v>0</v>
       </c>
       <c r="K21" s="15"/>
-      <c r="L21" s="18"/>
-      <c r="M21" s="16"/>
-    </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A22" s="15" t="str">
+      <c r="L21" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M21" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="15">
         <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
-        <v/>
-      </c>
-      <c r="B22" s="14"/>
-      <c r="C22" s="13"/>
-      <c r="D22" s="15"/>
+        <v>20</v>
+      </c>
+      <c r="B22" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E22" s="15"/>
       <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
+      <c r="G22" s="15">
+        <v>15</v>
+      </c>
       <c r="H22" s="15"/>
       <c r="I22" s="3"/>
       <c r="J22" s="15">
@@ -1520,20 +1823,32 @@
         <v>0</v>
       </c>
       <c r="K22" s="15"/>
-      <c r="L22" s="18"/>
-      <c r="M22" s="16"/>
-    </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A23" s="15" t="str">
+      <c r="L22" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M22" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="15">
         <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
-        <v/>
-      </c>
-      <c r="B23" s="14"/>
-      <c r="C23" s="13"/>
-      <c r="D23" s="15"/>
+        <v>21</v>
+      </c>
+      <c r="B23" s="14" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E23" s="15"/>
       <c r="F23" s="15"/>
-      <c r="G23" s="15"/>
+      <c r="G23" s="15">
+        <v>6</v>
+      </c>
       <c r="H23" s="15"/>
       <c r="I23" s="3"/>
       <c r="J23" s="15">
@@ -1541,20 +1856,32 @@
         <v>0</v>
       </c>
       <c r="K23" s="15"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="16"/>
-    </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A24" s="15" t="str">
+      <c r="L23" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M23" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A24" s="15">
         <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
-        <v/>
-      </c>
-      <c r="B24" s="14"/>
-      <c r="C24" s="13"/>
-      <c r="D24" s="15"/>
+        <v>22</v>
+      </c>
+      <c r="B24" s="14" t="s">
+        <v>74</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E24" s="15"/>
       <c r="F24" s="15"/>
-      <c r="G24" s="15"/>
+      <c r="G24" s="15">
+        <v>1</v>
+      </c>
       <c r="H24" s="15"/>
       <c r="I24" s="3"/>
       <c r="J24" s="15">
@@ -1562,20 +1889,32 @@
         <v>0</v>
       </c>
       <c r="K24" s="15"/>
-      <c r="L24" s="18"/>
-      <c r="M24" s="16"/>
-    </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A25" s="15" t="str">
+      <c r="L24" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M24" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A25" s="15">
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
-        <v/>
-      </c>
-      <c r="B25" s="14"/>
-      <c r="C25" s="13"/>
-      <c r="D25" s="15"/>
+        <v>23</v>
+      </c>
+      <c r="B25" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E25" s="15"/>
       <c r="F25" s="15"/>
-      <c r="G25" s="15"/>
+      <c r="G25" s="15">
+        <v>3</v>
+      </c>
       <c r="H25" s="15"/>
       <c r="I25" s="3"/>
       <c r="J25" s="15">
@@ -1583,20 +1922,32 @@
         <v>0</v>
       </c>
       <c r="K25" s="15"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="16"/>
-    </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A26" s="15" t="str">
+      <c r="L25" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A26" s="15">
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
-        <v/>
-      </c>
-      <c r="B26" s="14"/>
-      <c r="C26" s="13"/>
-      <c r="D26" s="15"/>
+        <v>24</v>
+      </c>
+      <c r="B26" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>30</v>
+      </c>
       <c r="E26" s="15"/>
       <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
+      <c r="G26" s="15">
+        <v>3</v>
+      </c>
       <c r="H26" s="15"/>
       <c r="I26" s="3"/>
       <c r="J26" s="15">
@@ -1604,19 +1955,309 @@
         <v>0</v>
       </c>
       <c r="K26" s="15"/>
-      <c r="L26" s="18"/>
-      <c r="M26" s="16"/>
+      <c r="L26" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M26" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A27" s="15">
+        <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
+        <v>25</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>80</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15">
+        <v>3</v>
+      </c>
+      <c r="H27" s="15"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="15">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="K27" s="15"/>
+      <c r="L27" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A28" s="15">
+        <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
+        <v>26</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E28" s="15"/>
+      <c r="F28" s="15"/>
+      <c r="G28" s="15">
+        <v>1</v>
+      </c>
+      <c r="H28" s="15"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="15">
+        <f t="shared" ref="J28:J35" si="1">(G28*E28)+F28</f>
+        <v>0</v>
+      </c>
+      <c r="K28" s="15"/>
+      <c r="L28" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A29" s="15">
+        <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
+        <v>27</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="D29" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15">
+        <v>1</v>
+      </c>
+      <c r="H29" s="15"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K29" s="15"/>
+      <c r="L29" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M29" s="16" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A30" s="15">
+        <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
+        <v>28</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D30" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15">
+        <v>4</v>
+      </c>
+      <c r="H30" s="15"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K30" s="15"/>
+      <c r="L30" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M30" s="16"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="15">
+        <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
+        <v>29</v>
+      </c>
+      <c r="B31" s="25" t="s">
+        <v>96</v>
+      </c>
+      <c r="C31" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15">
+        <v>4</v>
+      </c>
+      <c r="H31" s="15"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K31" s="15"/>
+      <c r="L31" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M31" s="16"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="15">
+        <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
+        <v>30</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>87</v>
+      </c>
+      <c r="C32" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>18</v>
+      </c>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15">
+        <v>4</v>
+      </c>
+      <c r="H32" s="15"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K32" s="15"/>
+      <c r="L32" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M32" s="16"/>
+    </row>
+    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A33" s="15">
+        <f>IF(B33&lt;&gt;"",COUNTA($B$3:B33),"")</f>
+        <v>31</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="C33" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15">
+        <v>1</v>
+      </c>
+      <c r="H33" s="15"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K33" s="15"/>
+      <c r="L33" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M33" s="16"/>
+    </row>
+    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A34" s="15">
+        <f>IF(B34&lt;&gt;"",COUNTA($B$3:B34),"")</f>
+        <v>32</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="C34" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15">
+        <v>1</v>
+      </c>
+      <c r="H34" s="15"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K34" s="15"/>
+      <c r="L34" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M34" s="16"/>
+    </row>
+    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A35" s="15">
+        <f>IF(B35&lt;&gt;"",COUNTA($B$3:B35),"")</f>
+        <v>33</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C35" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15">
+        <v>1</v>
+      </c>
+      <c r="H35" s="15"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="15">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="K35" s="15"/>
+      <c r="L35" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M35" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="F8:F9"/>
   </mergeCells>
-  <conditionalFormatting sqref="L3 L6 L11:L26">
+  <phoneticPr fontId="6" type="noConversion"/>
+  <conditionalFormatting sqref="L3 L6">
     <cfRule type="expression" priority="1">
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L5 L7:L10">
+  <conditionalFormatting sqref="L4:L5 L7:L35">
     <cfRule type="expression" priority="3">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -1633,19 +2274,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D26</xm:sqref>
+          <xm:sqref>D3:D35</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D191F27-4E1E-4078-9DF4-BD7DE8468C2E}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H26</xm:sqref>
+          <xm:sqref>H3:H35</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L26</xm:sqref>
+          <xm:sqref>L3:L35</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1656,9 +2297,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="19" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
Fillet and added servo shaft
</commit_message>
<xml_diff>
--- a/1_ORGO-15_P1/BOM_ORGO-15_P1.xlsx
+++ b/1_ORGO-15_P1/BOM_ORGO-15_P1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ORGOfly\ORGOfly-CAD-model\1_ORGO-15_P1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Drones\ORGOfly-CAD-model\1_ORGO-15_P1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D224F16-787E-44F1-8222-97A5CC2797A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9E55C83-D6FA-4264-88DD-62D087519179}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="127">
   <si>
     <t>#</t>
   </si>
@@ -408,13 +408,25 @@
   </si>
   <si>
     <t>4-7 days</t>
+  </si>
+  <si>
+    <t>Servo to Shaft Coupler (H25T Spline, 1/4" Bore)</t>
+  </si>
+  <si>
+    <t>1/4" D-Shaft (Stainless Steel, 1-1/2" Length)</t>
+  </si>
+  <si>
+    <t>https://eu.robotshop.com/products/servocity-1-4-d-shaft-stainless-steel-1-1-2-length?qd=e475ba9145954a5b0572979a4c1a9dfa</t>
+  </si>
+  <si>
+    <t>https://eu.robotshop.com/products/servo-to-shaft-coupler-h25t-spline-1-4-inch-bore?qd=888300ea906a262b32fb5f85def28ba5</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -550,7 +562,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -612,6 +624,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -954,12 +970,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="33.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="15">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -970,7 +986,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -981,7 +997,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -992,7 +1008,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -1003,7 +1019,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1014,7 +1030,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.25">
       <c r="C7" t="s">
         <v>13</v>
       </c>
@@ -1022,37 +1038,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.25">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1064,31 +1080,31 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:M28"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:M30"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.75" style="7" customWidth="1"/>
-    <col min="3" max="3" width="57.75" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.75" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="7" width="8.875" style="1"/>
-    <col min="8" max="8" width="4.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.25" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.875" style="1"/>
+    <col min="2" max="2" width="37.7109375" style="7" customWidth="1"/>
+    <col min="3" max="3" width="57.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="37.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="8.85546875" style="1"/>
+    <col min="8" max="8" width="4.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.28515625" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" style="1"/>
     <col min="13" max="13" width="48" style="17" customWidth="1"/>
-    <col min="14" max="16384" width="8.875" style="2"/>
+    <col min="14" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="15">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:13" ht="27" customHeight="1">
+    <row r="2" spans="1:13" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -1129,7 +1145,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="3" spans="1:13">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -1166,7 +1182,7 @@
       </c>
       <c r="M3" s="16"/>
     </row>
-    <row r="4" spans="1:13">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
@@ -1209,7 +1225,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="5" spans="1:13">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
@@ -1252,7 +1268,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:13">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
@@ -1295,7 +1311,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="7" spans="1:13">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
@@ -1338,7 +1354,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="8" spans="1:13">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
@@ -1381,7 +1397,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="9" spans="1:13">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
@@ -1420,7 +1436,7 @@
       </c>
       <c r="M9" s="16"/>
     </row>
-    <row r="10" spans="1:13" ht="42.75">
+    <row r="10" spans="1:13" ht="45" x14ac:dyDescent="0.25">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
@@ -1463,7 +1479,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="15">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
@@ -1494,7 +1510,7 @@
       </c>
       <c r="M11" s="16"/>
     </row>
-    <row r="12" spans="1:13">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A12" s="15">
         <f>IF(B12&lt;&gt;"",COUNTA($B$3:B12),"")</f>
         <v>10</v>
@@ -1535,7 +1551,7 @@
       </c>
       <c r="M12" s="16"/>
     </row>
-    <row r="13" spans="1:13">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A13" s="15">
         <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
         <v>11</v>
@@ -1578,7 +1594,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="14" spans="1:13">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A14" s="15">
         <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
         <v>12</v>
@@ -1609,7 +1625,7 @@
       </c>
       <c r="M14" s="16"/>
     </row>
-    <row r="15" spans="1:13">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A15" s="15">
         <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
         <v>13</v>
@@ -1640,7 +1656,7 @@
       </c>
       <c r="M15" s="16"/>
     </row>
-    <row r="16" spans="1:13">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A16" s="15">
         <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
         <v>14</v>
@@ -1681,7 +1697,7 @@
       </c>
       <c r="M16" s="16"/>
     </row>
-    <row r="17" spans="1:13">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A17" s="15">
         <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
         <v>15</v>
@@ -1724,7 +1740,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:13">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A18" s="15">
         <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
         <v>16</v>
@@ -1755,7 +1771,7 @@
       </c>
       <c r="M18" s="16"/>
     </row>
-    <row r="19" spans="1:13">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A19" s="15">
         <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
         <v>17</v>
@@ -1798,7 +1814,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="1:13">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A20" s="15">
         <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
         <v>18</v>
@@ -1841,7 +1857,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="21" spans="1:13">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A21" s="15">
         <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
         <v>19</v>
@@ -1884,7 +1900,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="22" spans="1:13">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A22" s="15">
         <v>19</v>
       </c>
@@ -1924,7 +1940,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="12.75" customHeight="1">
+    <row r="23" spans="1:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="15">
         <v>19</v>
       </c>
@@ -1964,7 +1980,7 @@
       </c>
       <c r="M23" s="16"/>
     </row>
-    <row r="24" spans="1:13" ht="15">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A24" s="15">
         <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
         <v>22</v>
@@ -1995,7 +2011,7 @@
       </c>
       <c r="M24" s="16"/>
     </row>
-    <row r="25" spans="1:13">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A25" s="15">
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
         <v>23</v>
@@ -2038,7 +2054,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="26" spans="1:13">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A26" s="15">
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
         <v>24</v>
@@ -2079,7 +2095,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="27" spans="1:13">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A27" s="15">
         <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
         <v>25</v>
@@ -2122,7 +2138,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="28" spans="1:13">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A28" s="15">
         <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
         <v>26</v>
@@ -2152,6 +2168,72 @@
         <v>36</v>
       </c>
       <c r="M28" s="16"/>
+    </row>
+    <row r="29" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A29" s="15">
+        <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
+        <v>27</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="13"/>
+      <c r="D29" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E29" s="15"/>
+      <c r="F29" s="15"/>
+      <c r="G29" s="15">
+        <v>4</v>
+      </c>
+      <c r="H29" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I29" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="J29" s="15">
+        <f t="shared" ref="J29" si="2">(G29*E29)+F29</f>
+        <v>0</v>
+      </c>
+      <c r="K29" s="15"/>
+      <c r="L29" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M29" s="16"/>
+    </row>
+    <row r="30" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="A30" s="15">
+        <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
+        <v>28</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>124</v>
+      </c>
+      <c r="C30" s="13"/>
+      <c r="D30" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15">
+        <v>4</v>
+      </c>
+      <c r="H30" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I30" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="J30" s="15">
+        <f t="shared" ref="J30" si="3">(G30*E30)+F30</f>
+        <v>0</v>
+      </c>
+      <c r="K30" s="15"/>
+      <c r="L30" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M30" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2163,7 +2245,7 @@
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L28">
+  <conditionalFormatting sqref="L4:L30">
     <cfRule type="expression" priority="3">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -2180,19 +2262,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D28</xm:sqref>
+          <xm:sqref>D3:D30</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D191F27-4E1E-4078-9DF4-BD7DE8468C2E}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H28</xm:sqref>
+          <xm:sqref>H3:H30</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L28</xm:sqref>
+          <xm:sqref>L3:L30</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2203,9 +2285,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="19"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed aileron to servo connection
</commit_message>
<xml_diff>
--- a/1_ORGO-15_P1/BOM_ORGO-15_P1.xlsx
+++ b/1_ORGO-15_P1/BOM_ORGO-15_P1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Drones\ORGOfly-CAD-model\1_ORGO-15_P1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9ED41114-CB5A-4C95-BC6E-3CB2DB657E89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5459295-ABFB-4924-90A9-B4DB8B5C86F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="133">
   <si>
     <t>#</t>
   </si>
@@ -410,29 +410,41 @@
     <t>4-7 days</t>
   </si>
   <si>
-    <t>Servo to Shaft Coupler (H25T Spline, 1/4" Bore)</t>
-  </si>
-  <si>
-    <t>1/4" D-Shaft (Stainless Steel, 1-1/2" Length)</t>
-  </si>
-  <si>
-    <t>https://eu.robotshop.com/products/servocity-1-4-d-shaft-stainless-steel-1-1-2-length?qd=e475ba9145954a5b0572979a4c1a9dfa</t>
-  </si>
-  <si>
-    <t>https://eu.robotshop.com/products/servo-to-shaft-coupler-h25t-spline-1-4-inch-bore?qd=888300ea906a262b32fb5f85def28ba5</t>
-  </si>
-  <si>
     <t>Servo to Shaft Coupler</t>
   </si>
   <si>
     <t>Shaft</t>
+  </si>
+  <si>
+    <t>https://de.aliexpress.com/item/1005002809828245.html?spm=a2g0o.productlist.main.3.748eXfSsXfSs7Y&amp;algo_pvid=bd082ef1-520b-41ef-a3e1-2187c186d930&amp;algo_exp_id=bd082ef1-520b-41ef-a3e1-2187c186d930-2&amp;pdp_ext_f=%7B%22order%22%3A%2218%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.65%217.19%21%21%218.55%218.04%21%400b15834e17843741284825723e0efc%2112000022295201218%21sea%21DE%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3A23220bf0%3Bm03_new_user%3A-29895&amp;curPageLogUid=bsg7dXE6wM3i&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005002809828245%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>https://de.aliexpress.com/item/1005012043076003.html?spm=a2g0o.productlist.main.1.734akWubkWubS6&amp;algo_pvid=72a68408-40b7-4073-b1de-9a88b68bfd7d&amp;algo_exp_id=72a68408-40b7-4073-b1de-9a88b68bfd7d-0&amp;pdp_ext_f=%7B%22order%22%3A%2219%22%2C%22spu_best_type%22%3A%22price%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2111.45%216.99%21%21%2186.66%2152.86%21%402161390417843739759033324e100c%2112000057366562845%21sea%21DE%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3A23220bf0%3Bm03_new_user%3A-29895&amp;curPageLogUid=b41WCP6q7Yv6&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005012043076003%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>D-Shaft  5x60mm</t>
+  </si>
+  <si>
+    <t>Servo to Shaft Coupler  25T, 5mm Bore</t>
+  </si>
+  <si>
+    <t>D-Shaft  5x45mm</t>
+  </si>
+  <si>
+    <t>https://de.aliexpress.com/item/1005008084078658.html?spm=a2g0o.productlist.main.1.141fi6Rii6Rixp&amp;algo_pvid=20a221db-2b99-4b91-8b19-68befc329f31&amp;algo_exp_id=20a221db-2b99-4b91-8b19-68befc329f31-0&amp;pdp_ext_f=%7B%22order%22%3A%22411%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%215.03%215.16%21%21%2138.10%2139.05%21%402103081117843750175155863e0d5b%2112000046474978340%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895&amp;curPageLogUid=w2a4Ew33IG5l&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005008084078658%7C_p_origin_prod%3A&amp;gatewayAdapt=glo2deu</t>
+  </si>
+  <si>
+    <t>Flanged Bearings 5x8x2.5mm</t>
+  </si>
+  <si>
+    <t>Bearing come at 10 pcs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -483,6 +495,13 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -568,7 +587,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -628,14 +647,17 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1088,7 +1110,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:M30"/>
+  <dimension ref="A1:M32"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
@@ -1379,7 +1401,7 @@
       <c r="E8" s="15">
         <v>10.91</v>
       </c>
-      <c r="F8" s="25">
+      <c r="F8" s="26">
         <v>17.25</v>
       </c>
       <c r="G8" s="15">
@@ -1422,7 +1444,7 @@
       <c r="E9" s="15">
         <v>6</v>
       </c>
-      <c r="F9" s="26"/>
+      <c r="F9" s="27"/>
       <c r="G9" s="15">
         <v>1</v>
       </c>
@@ -2177,21 +2199,23 @@
       </c>
       <c r="M28" s="16"/>
     </row>
-    <row r="29" spans="1:13" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A29" s="15">
         <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
         <v>27</v>
       </c>
       <c r="B29" s="24" t="s">
+        <v>128</v>
+      </c>
+      <c r="C29" s="24" t="s">
         <v>123</v>
-      </c>
-      <c r="C29" s="24" t="s">
-        <v>127</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="15"/>
+      <c r="E29" s="28">
+        <v>6.99</v>
+      </c>
       <c r="F29" s="15"/>
       <c r="G29" s="15">
         <v>4</v>
@@ -2199,12 +2223,12 @@
       <c r="H29" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I29" s="27" t="s">
+      <c r="I29" s="25" t="s">
         <v>126</v>
       </c>
       <c r="J29" s="15">
         <f t="shared" ref="J29" si="2">(G29*E29)+F29</f>
-        <v>0</v>
+        <v>27.96</v>
       </c>
       <c r="K29" s="15"/>
       <c r="L29" s="18" t="s">
@@ -2212,40 +2236,116 @@
       </c>
       <c r="M29" s="16"/>
     </row>
-    <row r="30" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A30" s="15">
         <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
         <v>28</v>
       </c>
       <c r="B30" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="C30" s="24" t="s">
         <v>124</v>
-      </c>
-      <c r="C30" s="24" t="s">
-        <v>128</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="15"/>
+      <c r="E30" s="15">
+        <v>7.19</v>
+      </c>
       <c r="F30" s="15"/>
       <c r="G30" s="15">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H30" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I30" s="27" t="s">
+      <c r="I30" s="25" t="s">
         <v>125</v>
       </c>
       <c r="J30" s="15">
         <f t="shared" ref="J30" si="3">(G30*E30)+F30</f>
-        <v>0</v>
+        <v>14.38</v>
       </c>
       <c r="K30" s="15"/>
       <c r="L30" s="18" t="s">
         <v>36</v>
       </c>
       <c r="M30" s="16"/>
+    </row>
+    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A31" s="15">
+        <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
+        <v>29</v>
+      </c>
+      <c r="B31" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="C31" s="24" t="s">
+        <v>124</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E31" s="15">
+        <v>7.19</v>
+      </c>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15">
+        <v>2</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I31" s="25" t="s">
+        <v>125</v>
+      </c>
+      <c r="J31" s="15">
+        <f t="shared" ref="J31" si="4">(G31*E31)+F31</f>
+        <v>14.38</v>
+      </c>
+      <c r="K31" s="15"/>
+      <c r="L31" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M31" s="16"/>
+    </row>
+    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A32" s="15">
+        <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
+        <v>30</v>
+      </c>
+      <c r="B32" s="24" t="s">
+        <v>131</v>
+      </c>
+      <c r="C32" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="15">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15">
+        <v>1</v>
+      </c>
+      <c r="H32" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I32" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="J32" s="15">
+        <f t="shared" ref="J32" si="5">(G32*E32)+F32</f>
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="K32" s="15"/>
+      <c r="L32" s="18" t="s">
+        <v>36</v>
+      </c>
+      <c r="M32" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -2257,7 +2357,7 @@
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L30">
+  <conditionalFormatting sqref="L4:L32">
     <cfRule type="expression" priority="3">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -2274,19 +2374,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D30</xm:sqref>
+          <xm:sqref>D3:D32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8D191F27-4E1E-4078-9DF4-BD7DE8468C2E}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$6</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H30</xm:sqref>
+          <xm:sqref>H3:H32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L30</xm:sqref>
+          <xm:sqref>L3:L32</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>